<commit_message>
M2: map.sql-Import, Auswertung (Status/Deltas/Events), Distanz mit Wrap, Inaktiven-Suche und Detailseiten
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1110,6 +1110,106 @@
         </is>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Datenquelle</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>map.sql-Format verifiziert (echte Datei ts12.x1.europe): 16 Spalten, Zusatzspalten region/isCapital/isCity/hasHarbor/victoryPoints; Völker 1,2,3,5; keine Escapes</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Datenquelle</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Eigene Allianz „Human“ = allianceId 36 (180 Dörfer) → TRAVIAN_ALLIANCE_ID=36</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Snapshot = Tagesaggregat; Status inactive ab INACTIVE_DAYS Tagesständen ohne Zuwachs; Erstimport ohne Events</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Prozess</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>main als leerer Basis-Branch fehlte; Anlage von main per Branch-Kopie, Force-Push wurde vom Sicherheitsmodus blockiert → PR enthält M1+M2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Allianz-Gruppe: Typen pro Allianz, eigene Gruppe (OWN+ALLIED), Mitgliederabgleich, Filter in Inaktiven-Suche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1210,6 +1210,31 @@
         </is>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Allianz-Gruppe: Typen OWN/ALLIED/NAP/NEUTRAL/ENEMY; „eigene Gruppe“ = OWN+ALLIED gilt überall als eigene Allianz (Abgleich, Einladungen, Filter); Setzen durch ADMIN/SYSTEMADMIN</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
M3: Accounts, Rollen/Rechte, Verifizierung (Einladung, Umbenennungs-Code, manuell), Admin-UI, Audit-Log, E2E
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1235,6 +1235,156 @@
         </is>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Registrierung nur über eigene Route; Better-Auth-Sign-up per Hook gesperrt; Rolle/banned nicht vom Client setzbar</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Rechte</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SYSTEMADMIN-Adressen brauchen Setup-Code (SYSTEMADMIN_SETUP_CODE, Default AUTH_SECRET) — sonst könnte jeder die Admin-Mail vorab registrieren (kein E-Mail-Versand)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Rechte</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ADMIN vergibt/ändert nur Rollen unterhalb ADMIN; ADMINs ernennt nur SYSTEMADMIN; permissions.edit/roles.assign der Rolle ADMIN nur durch SYSTEMADMIN änderbar (Aussperr-Schutz)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Rechte</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Neues Recht alliances.classify (ADMIN); Karten-/Inaktiven-/Ereignisseiten verlangen map.view (GUEST hat es per Default)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Verifizierung</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Einladung, Umbenennungs-Code und manuelle Freigabe gelten nur für Spieler der eigenen Allianz-Gruppe (OWN+ALLIED)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>E2E mit Playwright (Chromium vorinstalliert); npm run e2e getrennt von npm run ci</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
UI an Screenflow angeglichen: Sidebar-Shell, Auth-Screens, Gast-Verifizierung, Inaktive, Admin-Tabs; Planungsdokumente v2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1026,17 +1026,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>M1-Gerüst umgesetzt: Next 15 + Prisma 6 + Tailwind 3 + Vitest 2; Custom Server `server.ts`; Worker im selben Image; Repo bleibt Monorepo (Abweichung vom 5-Repo-Template)</t>
+          <t>Screenflow als eigenständige HTML-Datei für Claude Code (11 Screens inkl. Login, Einladung, Gast-Verifizierung, Chat-Anhänge/Lightbox; zuschaltbare CC-Hinweise)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+          <t>https://claude.ai/chat/3f8396b4-1960-410b-9762-e96c8eb5b39c</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1051,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Prozess</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Claude Code schreibt nicht nach Notion (CLAUDE.md-Direktive); Session-Row/Report läuft über projectos-reporter</t>
+          <t>M1-Gerüst umgesetzt: Next 15 + Prisma 6 + Tailwind 3 + Vitest 2; Custom Server `server.ts`; Worker im selben Image; Repo bleibt Monorepo (Abweichung vom 5-Repo-Template)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1076,12 +1076,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Datenquelle</t>
+          <t>Prozess</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>M2 blockiert: Sandbox-Netz verweigert ts12.x1.europe.travian.com (CONNECT 403) → echte map.sql-Fixture muss vom Nutzer geliefert werden</t>
+          <t>Claude Code schreibt nicht nach Notion (CLAUDE.md-Direktive); Session-Row/Report läuft über projectos-reporter</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1101,12 +1101,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Infra</t>
+          <t>Datenquelle</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Produktiv-Domain der App: humans-travian.com</t>
+          <t>M2 blockiert: Sandbox-Netz verweigert ts12.x1.europe.travian.com (CONNECT 403) → echte map.sql-Fixture muss vom Nutzer geliefert werden</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Datenquelle</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>map.sql-Format verifiziert (echte Datei ts12.x1.europe): 16 Spalten, Zusatzspalten region/isCapital/isCity/hasHarbor/victoryPoints; Völker 1,2,3,5; keine Escapes</t>
+          <t>Produktiv-Domain der App: humans-travian.com</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Eigene Allianz „Human“ = allianceId 36 (180 Dörfer) → TRAVIAN_ALLIANCE_ID=36</t>
+          <t>map.sql-Format verifiziert (echte Datei ts12.x1.europe): 16 Spalten, Zusatzspalten region/isCapital/isCity/hasHarbor/victoryPoints; Völker 1,2,3,5; keine Escapes</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1176,12 +1176,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Datenmodell</t>
+          <t>Datenquelle</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Snapshot = Tagesaggregat; Status inactive ab INACTIVE_DAYS Tagesständen ohne Zuwachs; Erstimport ohne Events</t>
+          <t>Eigene Allianz „Human“ = allianceId 36 (180 Dörfer) → TRAVIAN_ALLIANCE_ID=36</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1201,12 +1201,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Prozess</t>
+          <t>Datenmodell</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>main als leerer Basis-Branch fehlte; Anlage von main per Branch-Kopie, Force-Push wurde vom Sicherheitsmodus blockiert → PR enthält M1+M2</t>
+          <t>Snapshot = Tagesaggregat; Status inactive ab INACTIVE_DAYS Tagesständen ohne Zuwachs; Erstimport ohne Events</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1226,12 +1226,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Datenmodell</t>
+          <t>Prozess</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Allianz-Gruppe: Typen OWN/ALLIED/NAP/NEUTRAL/ENEMY; „eigene Gruppe“ = OWN+ALLIED gilt überall als eigene Allianz (Abgleich, Einladungen, Filter); Setzen durch ADMIN/SYSTEMADMIN</t>
+          <t>main als leerer Basis-Branch fehlte; Anlage von main per Branch-Kopie, Force-Push wurde vom Sicherheitsmodus blockiert → PR enthält M1+M2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Datenmodell</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Registrierung nur über eigene Route; Better-Auth-Sign-up per Hook gesperrt; Rolle/banned nicht vom Client setzbar</t>
+          <t>Allianz-Gruppe: Typen OWN/ALLIED/NAP/NEUTRAL/ENEMY; „eigene Gruppe“ = OWN+ALLIED gilt überall als eigene Allianz (Abgleich, Einladungen, Filter); Setzen durch ADMIN/SYSTEMADMIN</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Rechte</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SYSTEMADMIN-Adressen brauchen Setup-Code (SYSTEMADMIN_SETUP_CODE, Default AUTH_SECRET) — sonst könnte jeder die Admin-Mail vorab registrieren (kein E-Mail-Versand)</t>
+          <t>Registrierung nur über eigene Route; Better-Auth-Sign-up per Hook gesperrt; Rolle/banned nicht vom Client setzbar</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ADMIN vergibt/ändert nur Rollen unterhalb ADMIN; ADMINs ernennt nur SYSTEMADMIN; permissions.edit/roles.assign der Rolle ADMIN nur durch SYSTEMADMIN änderbar (Aussperr-Schutz)</t>
+          <t>SYSTEMADMIN-Adressen brauchen Setup-Code (SYSTEMADMIN_SETUP_CODE, Default AUTH_SECRET) — sonst könnte jeder die Admin-Mail vorab registrieren (kein E-Mail-Versand)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Neues Recht alliances.classify (ADMIN); Karten-/Inaktiven-/Ereignisseiten verlangen map.view (GUEST hat es per Default)</t>
+          <t>ADMIN vergibt/ändert nur Rollen unterhalb ADMIN; ADMINs ernennt nur SYSTEMADMIN; permissions.edit/roles.assign der Rolle ADMIN nur durch SYSTEMADMIN änderbar (Aussperr-Schutz)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1351,12 +1351,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Verifizierung</t>
+          <t>Rechte</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Einladung, Umbenennungs-Code und manuelle Freigabe gelten nur für Spieler der eigenen Allianz-Gruppe (OWN+ALLIED)</t>
+          <t>Neues Recht alliances.classify (ADMIN); Karten-/Inaktiven-/Ereignisseiten verlangen map.view (GUEST hat es per Default)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1376,15 +1376,165 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>Verifizierung</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Einladung, Umbenennungs-Code und manuelle Freigabe gelten nur für Spieler der eigenen Allianz-Gruppe (OWN+ALLIED)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>E2E mit Playwright (Chromium vorinstalliert); npm run e2e getrennt von npm run ci</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Screenflow (docs/ui/screenflow.html) ist verbindlich; M1–M3-UI wurde nachträglich daran angeglichen (Sidebar-Shell, Tokens, Auth-Screens, Admin-Tabs, Inaktive)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Admin hat zusätzlich zu den 3 Tabs der Vorlage die Tabs Allianzen (Allianz-Gruppe), Konten und Audit-Log</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SMTP wird eingeplant (Passwort vergessen / Reset); bis dahin /forgot mit Hinweis</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TRAVIAN_ALLIANCE_ID ist nur Startwert (implizit OWN); weitere Allianzen der Gruppe werden im Admin-UI markiert</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Verifizierung</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>„IGM-Text kopieren“ erzeugt einen neuen Link (alter wird widerrufen), weil nur der Token-Hash gespeichert wird; Text einmalig sichtbar</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>
@@ -1415,6 +1565,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
M4: Chat (Kanäle, Sammelraum, Tags, Task-Forces, Realtime, Anhänge mit Vorschau/Lightbox, Suche, Admin-Tab), Systemschriften
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1535,6 +1535,181 @@
         </is>
       </c>
       <c r="E44" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Keine externen Fonts (DSGVO): Systemschriften (Arial/Georgia/Courier) statt Google Fonts</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>GUEST erhält chat.read; welche Kanäle ein Gast sieht, steuert minReadRole (Standard: nur Mixed topics)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Nachrichtentext wird als Markdown-Quelltext gespeichert und beim Rendern in React-Knoten übersetzt (kein HTML, keine Sanitizer-Abhängigkeit)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Volltextsuche über GIN-Ausdrucksindex statt generierter tsvector-Spalte (vermeidet Prisma-Drift)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Task-Force-Verwaltung: Leads, taskforce.manage und Admins; letzter Lead nicht entfernbar; Nicht-Mitglieder bekommen 404 statt 403 auf Task-Force-Seiten</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>PDF-Seitenvorschau per pdftoppm (poppler-utils im Docker-Image); ohne das Tool zeigt die PDF-Karte keinen Seitenvorschau</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Kanal-Rechte: Kanäle verwalten = settings.edit, Tags = tags.manage</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
SMTP: Passwort-Reset per E-Mail (/forgot, /reset-password)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1710,6 +1710,31 @@
         </is>
       </c>
       <c r="E51" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>SMTP umgesetzt: Passwort-Reset per E-Mail (nodemailer); E-Mail-Verifizierung bei Registrierung bewusst noch nicht aktiviert</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
M5 + Phase-2-Gerüst: Meine Dörfer, KI-Instruktionen, Erinnerungen, Screenshot-Upload (Stub), Spieldaten-Schema und -Seite
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1735,6 +1735,106 @@
         </is>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>VillageState ist eine Zeile je Dorf (aktueller Ist-Zustand) mit Zeitstempeln je Bereich; Verlauf/Historie bewusst noch nicht</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Datenquelle</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Spieldaten-Analyse (Schritt 1) blockiert: Travian-Wissensdatenbank aus der Sandbox nicht erreichbar → Netzfreigabe oder HAR/Export nötig</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>KI</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>AiClient/ScreenshotPipeline/Advisor nur als Stubs; Screenshots werden gespeichert, Erkennung inaktiv; keine echten Claude-Calls</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>„Meine Dörfer“ öffnet das Dorf-Dashboard des größten Dorfs; Übersicht zeigt Dörfertabelle; Spieler ohne verifizierten Spieler sehen Hinweis + Link zur Verknüpfung</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Betrieb: mehrere Allianz-IDs, Weltende-Erkennung + Neue Welt, Pruning, Spieldaten-Importformat/Probe, Docker-Fix, Backup/Deploy-Skripte, DEPLOY.md, docs/reports
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1835,6 +1835,131 @@
         </is>
       </c>
       <c r="E56" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TRAVIAN_ALLIANCE_ID akzeptiert mehrere IDs (kommagetrennt); alle gelten als „Eigene Allianz“</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Betrieb</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Weltende: 36 fehlgeschlagene stündliche map.sql-Importe in Folge → Welt „beendet“ (Archivmodus, Auto-Reset bei Erfolg); Neue Welt per scripts/new-world.ts (Konten/Chat bleiben, Member → Gast)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Datenquelle</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Wissensdatenbank: Analyse-Skript läuft auf dem Server (Entwicklungsumgebung ohne Zugriff); halbjährlicher Scraper vorgesehen, sobald Struktur + Erlaubnis von Travian Games geklärt (Auftrag sah nur manuellen Import vor)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Betrieb</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>map.sql-Abruf stündlich geprüft, Import nur bei geändertem Hash (täglich); Dorf-Rohzeilen nur für die letzten 3 Snapshots, Verlauf bleibt in PlayerDailyStat</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Betrieb</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Reports unter docs/reports (technical.md, changelog.md) statt Session-Report nach projectos-reporter</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Truppenübersicht für Admins/Moderatoren (troops.view), manuelle Truppeneingabe, Transparenzhinweise
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1960,6 +1960,81 @@
         </is>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rechte</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Neues Recht troops.view (Truppen aller Mitglieder einsehen): Moderator + Admin per Default, in der Rechte-Matrix änderbar</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Datenschutz</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Truppen-Einsicht ist für Mitglieder transparent (Hinweis auf Einladungsseite und im Dorf-Dashboard) und wird im Audit-Log protokolliert</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Datenmodell</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Truppendaten bis zur aktiven Screenshot-Erkennung per manueller Eingabe (VillageState.troops, Zeitstempel troopsAt)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Screenshot-Erkennung: Claude Vision, Konfidenzprüfungen, Lernmodus + Review-UI, Eval-Skript, 14 Muster mit Gold-Daten
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2035,6 +2035,131 @@
         </is>
       </c>
       <c r="E64" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung: Claude Vision mit Structured Outputs statt klassischem OCR; ein einheitliches Lesungsformat (lib/ai/reading.ts) für alle Arten; Modell per ANTHROPIC_MODEL (Default claude-opus-5-5)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Konfidenz = deterministische Prüfungen (Summenzeilen, Spaltenzahl, Koordinaten, eigene Dörfer) × Konsens aus VISION_PASSES Durchläufen, gedeckelt durch KI-Selbstauskunft; nie nur die KI-Selbstauskunft</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Lernmodus: Bestätigung/Korrektur im UI (/screenshots) speichert Bild + richtige Lesung als Few-Shot-Beispiel (VisionExample, je Art max. 30, 1 je Art im Prompt); Auto-Übernahme erst nach VISION_LEARNING_MIN Bestätigungen je Art und Konfidenz ≥ VISION_AUTO_ACCEPT</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Desktop-Statistiktabellen nennen nur Dorfnamen → Zuordnung zu eigenen Dörfern per Name; Lagersummen mit 1 % Toleranz (Bestände ticken), Produktion exakt; Desktop-Produktion = brutto, Seitenleiste/Mobil = netto</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Screenshot-Erkennung</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Screenshot-Fixtures + Gold-JSON in tests/fixtures/screenshots; Güte messbar mit scripts/eval-vision.ts (braucht API-Key)</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Tag-Typen (Achsen) an Kanäle gebunden; E2E an neue Konten-/Upload-Texte angepasst
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2160,6 +2160,31 @@
         </is>
       </c>
       <c r="E69" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Tag-Typen (Achsen) an Kanäle gebunden: n:m Zuweisung, je Typ Einzel-/Mehrfachauswahl (Default ein Tag) und Pflicht-Schalter; bestehende Tags im Typ „Kategorie“</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Allianz-Schedule: Calls aus Vorlagen (Koordinaten → Spieler/Dorf/Link), geplant oder auf Abruf, Rechte schedule.view/manage
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2185,6 +2185,56 @@
         </is>
       </c>
       <c r="E70" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Allianz-Schedule: Calls aus Vorlagen, Ziel per Koordinate aus map.sql, Zeitplan im Server-Prozess (30 s), Link zur Spielerseite; Rechte schedule.view/manage</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Planung</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Reihenfolge der neuen Features: 1 Schedule, 2 Task-Force (Einladung mit Annahme, 4 Rollen: Gründer/Lead/Mitglied/Leser, Rollenvergabe nur Gründer), 3 Messenger (DM für alle, Rundnachricht ab Moderator)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Task-Forces: Einladung mit Annahme, Rollen Gründer/Lead/Mitglied/Leser, Rollenvergabe nur durch Gründer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2235,6 +2235,31 @@
         </is>
       </c>
       <c r="E72" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Task-Forces</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Einladung mit Annahme, Rollen Gründer/Lead/Mitglied/Leser; nur Gründer (Admin als Notausgang) vergibt Rollen und archiviert; Ersteller = Gründer, nicht entfernbar</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Messenger: Direktnachrichten und Rundnachrichten (getrennt von Kanälen), Ungelesen-Zähler, Live-Zustellung
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2260,6 +2260,31 @@
         </is>
       </c>
       <c r="E73" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Messenger</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Messenger getrennt von Kanälen: DM 1:1 für alle Mitglieder (Gäste nicht), Rundnachrichten ab Moderator mit Zielgruppen, Antwort per DM, Lesestatus für Absender; DMs unverschlüsselt (Hinweis nötig)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Screenshots: WebP-Komprimierung beim Upload, Aufbewahrungsfrist, Seite „Meine Bilder & Dateien“
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2285,6 +2285,56 @@
         </is>
       </c>
       <c r="E74" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Dateien</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Lokale Ablage (Docker-Volume, im Backup) statt S3 – Adapter bleibt austauschbar; Screenshots nur als WebP q88 voller Auflösung + Vorschau, Original wird verworfen; Aufbewahrung 30 Tage (Lern-Beispiele bleiben); Seite „Meine Bilder &amp; Dateien“</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Vision</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Structured-Output-Schema darf max. 16 Union-Parameter haben → Wire-Format mit Strings statt nullable-Typen, Konvertierung im Code</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Spieldaten: Vertrags-Invariante – Import nur für die eigene Welt (Host, Version, Geschwindigkeit)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2335,6 +2335,31 @@
         </is>
       </c>
       <c r="E76" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Spieldaten</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Vertrags-Invariante: Spieldaten nur für die eigene Welt (Host, Spielversion, Server-Geschwindigkeit); Abweichung = ganze Datei abgelehnt; keine Umrechnung; Scraper erst nach Probe + Genehmigung</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Spieldaten: Import der Gebäude aus der Legends-Wissensdatenbank (sicherer Literal-Parser, Welt-/Speed-Bindung)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2360,6 +2360,31 @@
         </is>
       </c>
       <c r="E77" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Spieldaten</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Wissensdatenbank-Daten stecken in main.js (SPA); wird per eigenem Literal-Parser gelesen, nie ausgeführt; Import Gebäude (Welt/Version/Speed-Bindung, Bauzeit auf Welt-Speed per Formel der Quelle); Truppen nicht enthalten</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Einheitennamen je Volk aus dem Support-Artikel (nur Namen), Benennung der Truppen über das Volk des Dorfbesitzers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2385,6 +2385,31 @@
         </is>
       </c>
       <c r="E78" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Spieldaten</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Einheitennamen nur aus dem offiziellen Support-Artikel (Namen je Volk/Platz); Kampfwerte/Zeiten/Crop-Wert nicht übernommen (Schmiede/Kaserne 20 bzw. unplausibel); Plätze 7–10 offen</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
UI: keine fremden E-Mails, Systemadmin als Admin anzeigen; i18n-Entscheidung dokumentiert
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2410,6 +2410,23 @@
         </is>
       </c>
       <c r="E79" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>E-Mails fremder Nutzer nie im FE; Systemadmin im UI als Admin; Englisch Basissprache/Pflicht für Beta</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
i18n: UI komplett zweisprachig (EN Basis, DE), Sprache pro Konto, Fehler über Schlüssel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2427,6 +2427,23 @@
         </is>
       </c>
       <c r="C80" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>i18n umgesetzt: Englisch Basis, Deutsch Übersetzung, Sprache pro Konto; Fehler über AppError-Schlüssel</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Spieldaten: Vorteile je Stufe + Vergleich, Truppennamen; S3-Bucket für Screenshots, 10-MB-Kontingent, Platzhalter für entfernte Chat-Dateien
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2444,6 +2444,23 @@
         </is>
       </c>
       <c r="C81" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Screenshots in eigenem S3-Bucket, 10 MB je Nutzer, Löschen hinterlässt Chat-Platzhalter; Vorteile je Stufe über zentrale Effekt-Registry</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Registrierung nur für Gruppe/enge Bündnispartner, Sperre bis zur Verifizierung, Knopf „Verlinkung nachweisen“
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2461,6 +2461,23 @@
         </is>
       </c>
       <c r="C82" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Registrierung nur für Gruppe + Typ Enge Bündnispartner; GUEST gesperrt bis Verifizierung; Nachweis-Knopf mit map.sql-Abruf (max. alle 5 min); Bündnispartner werden nach Verifizierung MEMBER (eigene Rolle mit weniger Rechten = möglicher Folgeschritt)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Menü verschlankt (Untermenüs Dörfer/Chats/Admin, OCR-Scans), E-Mail-Bestätigung bei aktivem SMTP, Konten-Hinweis bereinigt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2478,6 +2478,81 @@
         </is>
       </c>
       <c r="C83" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>79</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Menü verschlankt: Übersicht mit Dörfer-Untermenü (statt „Meine Dörfer“), „Inaktivensuche“, „Chats“ mit Kanälen + Task-Forces als Untermenü, Schedule/Truppen unter Admin (für Konten ohne Admin-Bereich weiter Hauptpunkt), „OCR-Scans“ statt „Screenshots“</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>80</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Dynamischer Loader als Spinner am Link (useLinkStatus) statt loading.tsx – loading.tsx brach Server-Action-Weiterleitungen auf derselben Seite und den 404-Status</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>81</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>E-Mail-Bestätigung als Freigabe-Kriterium, nur aktiv wenn SMTP_HOST gesetzt; Bestandskonten per Migration als bestätigt; Notzugang ausgenommen; Passwort-Reset per Mail bestand bereits</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Mein Konto mit Passwort-Reset-Link; Image ohne Backups/Cache, Deploy räumt Speicher auf
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2553,6 +2553,56 @@
         </is>
       </c>
       <c r="E86" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>82</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Seite „Mein Konto“ mit Reset-Link an eigene Adresse; Reset-Seite bleibt außerhalb des App-Layouts (/reset-password)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>83</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Betrieb</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Backups/Laufzeitdaten nie im Docker-Image (.dockerignore); deploy.sh räumt Build-Cache vor jedem Build auf; SMTP über Port 465 (implizites TLS), da Plesk 587 nicht anbietet</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
KI-Vorschläge Phase 1: Lagebild, Tageslauf mit Kostendeckel, Nutzungsprotokoll, Dorftyp, Rechte, Admin-Tab KI & Kosten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2603,6 +2603,81 @@
         </is>
       </c>
       <c r="E88" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>84</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>KI</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Advisor und Incidents mit Haiku 5.5; Monatsbudget 15 € inkl. S3 variabel (Hetzner-Fixum nicht eingerechnet); 1×/Tag per Knopf, Lagebild deterministisch, KI nur Priorisierung mit fester JSON-Struktur</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>85</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Rechte</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ai.advice/incidents.report für Mitglieder, Gäste per Rechte-Matrix freigebbar; ohne Recht keine Prompt-Felder; Incidents aller sehen nur Admins</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>86</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>KI</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Suche im Verlauf zuerst per Postgres-Volltextsuche statt Vektoren</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Incidents: Kampfbericht oder manuell melden, Bedrohungsmodus, Lagebewertung, Hilfe im Deff-Call, Admin-Übersicht
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2678,6 +2678,31 @@
         </is>
       </c>
       <c r="E91" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>87</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Incidents</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Eigene Seite mit Erklärung; Bedrohungsmodus 3 Tage (1 ohne weitere Angriffe); Hilfe-Anfrage als englische Nachricht im Deff-Call; ein zusätzlicher KI-Lauf je Incident</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Gedächtnis: Volltextsuche mit hartem Nutzerfilter und Row-Level Security, im Lagebild und als Verlaufssuche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,31 @@
         </is>
       </c>
       <c r="E92" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>88</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sicherheit</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Gedächtnis-Suche: expliziter Nutzerfilter in jeder Abfrage + Row-Level Security unter eigener DB-Rolle ally_memory (App-User ist Superuser, RLS sonst wirkungslos)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Öffentliche Hilfeseite mit aufklappbaren Punkten je Funktion, Quicklinks mit Login-Rücksprung und Kurzvideos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2728,6 +2728,31 @@
         </is>
       </c>
       <c r="E93" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>89</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Hilfe</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Öffentliche Hilfeseite ohne Login; Quicklinks nur nach Login (Rücksprung per next); vier Bereiche mit aufklappbaren Punkten je Funktion; Kurzvideos per Playwright-Aufnahme</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Ein Weg vom Incident zum Call (Recht je Call-Typ), Hilfe: Kacheln mit Einzelansicht, Weg A/B, Datenfluss-Skizze
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2753,6 +2753,56 @@
         </is>
       </c>
       <c r="E94" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>90</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Incidents/Calls</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Ein Weg: Hilfe anfragen erzeugt einen echten Call, wenn die Rolle den Call-Typ aus Incidents darf (Recht je Call-Typ, im Schedule einstellbar); sonst kurze Deff-Call-Nachricht. „Push“ = Direktnachricht laut Vorlage</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>91</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Hilfe</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Kacheln als Buttons mit Einzelansicht je Bereich; Einstieg als Weg A/B; Datenfluss-Skizze (A/B1/B2, Incidents, Truppen nur Admins/Moderatoren)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Fix empty 'Bis:' in incident calls; overview PDF (EN/DE) at /help/pdf
- Incident call uses threat-mode end as event time
- renderCall drops lines whose placeholders are all empty
- Public /help/pdf serves public/help/overview.<lang>.pdf, linked from /help

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2803,6 +2803,56 @@
         </is>
       </c>
       <c r="E96" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>92</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Calls</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>„Bis“ im Call aus einem Incident = Ende des Bedrohungsmodus; Vorlagenzeilen, deren Platzhalter alle leer sind, entfallen ganz (keine leeren „Bis:“-Zeilen)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>93</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Hilfe</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Kurzübersicht als 5-seitiges PDF (EN/DE) öffentlich unter /help/pdf (?lang=de|en, sonst UI-Sprache); Link oben auf /help</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>

<commit_message>
Call templates in English: optional English text per template
- CallTemplate.bodyEn / AllianceCall.templateEn (migration fills defaults if unchanged)
- Channel message in sender's language, DMs and mails per recipient
- Schedule: English text field, preview in UI language

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM
</commit_message>
<xml_diff>
--- a/docs/projectos/entscheidungen.xlsx
+++ b/docs/projectos/entscheidungen.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2853,6 +2853,31 @@
         </is>
       </c>
       <c r="E98" t="inlineStr">
+        <is>
+          <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>94</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Calls</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Call-Vorlagen zweisprachig: Text (Haupttext) + optional englischer Text. Kanal-Nachricht in der Sprache des Absenders, Direktnachrichten und Rundmails je Empfängersprache; Standardvorlagen per Migration ergänzt, wenn unverändert</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>https://claude.ai/code/session_01R8U6NZntnAU4Sd6J6QwApM</t>
         </is>

</xml_diff>